<commit_message>
Developed inventory_custom_fields.py script to inventory the custom fields in the Clio Templates.
</commit_message>
<xml_diff>
--- a/CustomField_LookupTable.xlsx
+++ b/CustomField_LookupTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft5071812-my.sharepoint.com/personal/tdolan_quillarrowlaw_com/Documents/Documents/ClioTemplates_CustomFields_MassUpdate/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="320" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71973B49-C4EF-44E7-956D-1A0CFE512676}"/>
+  <xr:revisionPtr revIDLastSave="321" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E602CCA5-E9A1-41A9-ABA2-6BDCA8B1D12A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
+    <workbookView xWindow="36750" yWindow="900" windowWidth="18660" windowHeight="13770" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
   </bookViews>
   <sheets>
     <sheet name="LookupTable" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
   <si>
     <t>New_Value</t>
   </si>
@@ -44,46 +44,46 @@
     <t>Old_Value</t>
   </si>
   <si>
-    <t>&lt;&lt; Matter.ResponsibleAttorney   &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;   MATTER.CUSTOMFIELD.PLAINTIFFSNAMESHORT &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;   Matter.CustomField.PlaintiffsFullLegalName   &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.CaseNumber&gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;Matter.CustomField.DefendantsFullLegalName &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;Matter.CustomField.Judge&gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.responsibleattorney.email &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.ResponsibleAttorney_Change1  &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;   MATTER.CUSTOMFIELD.PLAINTIFFSNAMESHORT_Change1   &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;   Matter.CustomField.PlaintiffsFullLegalName_Change1  &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.CaseNumber_Change1  &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;Matter.CustomField.DefendantsFullLegalName_Change1  &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;Matter.CustomField.Judge_Change1  &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.responsibleattorney.email_Change1  &gt;&gt;</t>
+    <t>&lt;&lt; Matter.ResponsibleAttorney &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.ResponsibleAttorney_UPDATED_030526 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.ResponsibleAttorney.JobTitle.Name &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.ResponsibleAttorney.JobTitle.Name_UPDATED_030526 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.PlaintiffsNameShort &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.PlaintiffsNameShort_UPDATED_030526 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; MATTER.CUSTOMFIELD.COUNTY &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; MATTER.CUSTOMFIELD.COUNTY_UPDATED_030526 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;Matter.CustomField.DateMatterFiled &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;Matter.CustomField.DateMatterFiled_UPDATED_030526 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.VehicleYear &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.VehicleYear_UPDATED_030526 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; User.Name &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; User.Name_UPDATED_030526 &gt;&gt;</t>
   </si>
 </sst>
 </file>
@@ -107,27 +107,15 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor theme="4" tint="0.79998168889431442"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="5">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -156,37 +144,9 @@
         <color indexed="64"/>
       </right>
       <top style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -195,7 +155,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -203,28 +163,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="5">
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
           <color indexed="64"/>
@@ -232,13 +184,35 @@
         <right style="medium">
           <color indexed="64"/>
         </right>
-        <top/>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
         <bottom style="thin">
           <color indexed="64"/>
         </bottom>
         <vertical/>
         <horizontal/>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -294,10 +268,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}" name="Table1" displayName="Table1" ref="A1:B8" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="A1:B8" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}" name="Table1" displayName="Table1" ref="A1:B10" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:B10" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{52BB13A1-40AB-4518-B0DE-62637CB7D74A}" name="Old_Value" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{52BB13A1-40AB-4518-B0DE-62637CB7D74A}" name="Old_Value" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{06BCDB60-C4F4-4E5F-B692-5B8737E55DE6}" name="New_Value" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -621,13 +595,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAF23435-C8D7-4BEB-89A9-D8A938A40D38}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="65.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -636,62 +610,84 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>9</v>
+      <c r="B2" s="3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>11</v>
+      <c r="A4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>12</v>
+        <v>6</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B8" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="6" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="7" t="s">
+      <c r="B10" s="4" t="s">
         <v>15</v>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="B3">
+    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B9">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
Added --normalize-case so uppercase/lowercase are counted together, updated verify_template_updates.py to strip mc:Fallback XML when using --deep-scan so we are not counting the same value twice.
</commit_message>
<xml_diff>
--- a/CustomField_LookupTable.xlsx
+++ b/CustomField_LookupTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft5071812-my.sharepoint.com/personal/tdolan_quillarrowlaw_com/Documents/Documents/ClioTemplates_CustomFields_MassUpdate/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="321" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E602CCA5-E9A1-41A9-ABA2-6BDCA8B1D12A}"/>
+  <xr:revisionPtr revIDLastSave="326" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A37C58DF-A8FC-4E46-994B-2BD81DAF039B}"/>
   <bookViews>
-    <workbookView xWindow="36750" yWindow="900" windowWidth="18660" windowHeight="13770" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
+    <workbookView xWindow="30360" yWindow="705" windowWidth="18570" windowHeight="13680" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
   </bookViews>
   <sheets>
     <sheet name="LookupTable" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>New_Value</t>
   </si>
@@ -44,46 +44,154 @@
     <t>Old_Value</t>
   </si>
   <si>
-    <t>&lt;&lt; Matter.ResponsibleAttorney &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.ResponsibleAttorney_UPDATED_030526 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.ResponsibleAttorney.JobTitle.Name &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.ResponsibleAttorney.JobTitle.Name_UPDATED_030526 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.PlaintiffsNameShort &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.PlaintiffsNameShort_UPDATED_030526 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; MATTER.CUSTOMFIELD.COUNTY &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; MATTER.CUSTOMFIELD.COUNTY_UPDATED_030526 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;Matter.CustomField.DateMatterFiled &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt;Matter.CustomField.DateMatterFiled_UPDATED_030526 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.VehicleYear &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.VehicleYear_UPDATED_030526 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; User.Name &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; User.Name_UPDATED_030526 &gt;&gt;</t>
+    <t>&lt;&lt; date.verbose &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; date.verbose _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.casenumber &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.casenumber _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.county &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.county _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.courtdepartment &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.courtdepartment _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.datematterfiled &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.datematterfiled _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.defendantsfulllegalname &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.defendantsfulllegalname _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.defendantsnameshort &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.defendantsnameshort _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.judge &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.judge _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.occitystatezip &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.occitystatezip _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.ocfirmname &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.ocfirmname _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.ocname1 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.ocname1 _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.ocname2 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.ocname2 _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.ocname3 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.ocname3 _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.ocstreetaddress &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.ocstreetaddress _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.plaintiffsfulllegalname &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.plaintiffsfulllegalname _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.plaintiffsnameshort &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.plaintiffsnameshort _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.trialdate.verbose &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.trialdate.verbose _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.vehiclemake &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.vehiclemake _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.vehicleyear &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.vehicleyear _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.vinnumber &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.vinnumber _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.responsibleattorney &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.responsibleattorney _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.responsibleattorney.email &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.responsibleattorney.email _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.responsibleattorney.jobtitle.name &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.responsibleattorney.jobtitle.name _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.responsibleattorney.name &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.responsibleattorney.name _UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; user.name &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; user.name _UPDATED_031126 &gt;&gt;</t>
   </si>
 </sst>
 </file>
@@ -115,7 +223,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -123,39 +231,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -163,37 +243,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="5">
-    <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -213,6 +267,25 @@
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="medium">
+          <color indexed="64"/>
+        </left>
+        <right style="medium">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -268,11 +341,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}" name="Table1" displayName="Table1" ref="A1:B10" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:B10" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}" name="Table1" displayName="Table1" ref="A1:B26" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:B26" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{52BB13A1-40AB-4518-B0DE-62637CB7D74A}" name="Old_Value" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{06BCDB60-C4F4-4E5F-B692-5B8737E55DE6}" name="New_Value" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{06BCDB60-C4F4-4E5F-B692-5B8737E55DE6}" name="New_Value" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -595,7 +668,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAF23435-C8D7-4BEB-89A9-D8A938A40D38}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="65.7109375" customWidth="1"/>
@@ -610,83 +683,211 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+      <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>7</v>
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>9</v>
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>11</v>
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>7</v>
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>13</v>
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>15</v>
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B24" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>48</v>
+      </c>
+      <c r="B25" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B3">
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B9">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Updated .gitignore to include verification_report.csv and added CHANGELOG_2026-03-12.txt
</commit_message>
<xml_diff>
--- a/CustomField_LookupTable.xlsx
+++ b/CustomField_LookupTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft5071812-my.sharepoint.com/personal/tdolan_quillarrowlaw_com/Documents/Documents/ClioTemplates_CustomFields_MassUpdate/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="326" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A37C58DF-A8FC-4E46-994B-2BD81DAF039B}"/>
+  <xr:revisionPtr revIDLastSave="329" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB76B858-04F5-4F69-8B88-067FEBBA2A04}"/>
   <bookViews>
-    <workbookView xWindow="30360" yWindow="705" windowWidth="18570" windowHeight="13680" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
+    <workbookView xWindow="32160" yWindow="1425" windowWidth="18570" windowHeight="13680" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
   </bookViews>
   <sheets>
     <sheet name="LookupTable" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>New_Value</t>
   </si>
@@ -62,30 +62,6 @@
     <t>&lt;&lt; matter.customfield.county _UPDATED_031126 &gt;&gt;</t>
   </si>
   <si>
-    <t>&lt;&lt; matter.customfield.courtdepartment &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.courtdepartment _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.datematterfiled &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.datematterfiled _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.defendantsfulllegalname &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.defendantsfulllegalname _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.defendantsnameshort &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.defendantsnameshort _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
     <t>&lt;&lt; matter.customfield.judge &gt;&gt;</t>
   </si>
   <si>
@@ -116,12 +92,6 @@
     <t>&lt;&lt; matter.customfield.ocname2 _UPDATED_031126 &gt;&gt;</t>
   </si>
   <si>
-    <t>&lt;&lt; matter.customfield.ocname3 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.ocname3 _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
     <t>&lt;&lt; matter.customfield.ocstreetaddress &gt;&gt;</t>
   </si>
   <si>
@@ -132,66 +102,6 @@
   </si>
   <si>
     <t>&lt;&lt; matter.customfield.plaintiffsfulllegalname _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.plaintiffsnameshort &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.plaintiffsnameshort _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.trialdate.verbose &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.trialdate.verbose _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.vehiclemake &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.vehiclemake _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.vehicleyear &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.vehicleyear _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.vinnumber &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.vinnumber _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.responsibleattorney &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.responsibleattorney _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.responsibleattorney.email &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.responsibleattorney.email _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.responsibleattorney.jobtitle.name &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.responsibleattorney.jobtitle.name _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.responsibleattorney.name &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.responsibleattorney.name _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; user.name &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; user.name _UPDATED_031126 &gt;&gt;</t>
   </si>
 </sst>
 </file>
@@ -341,8 +251,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}" name="Table1" displayName="Table1" ref="A1:B26" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:B26" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}" name="Table1" displayName="Table1" ref="A1:B11" totalsRowShown="0" headerRowDxfId="4">
+  <autoFilter ref="A1:B11" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{52BB13A1-40AB-4518-B0DE-62637CB7D74A}" name="Old_Value" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{06BCDB60-C4F4-4E5F-B692-5B8737E55DE6}" name="New_Value" dataDxfId="2"/>
@@ -668,7 +578,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAF23435-C8D7-4BEB-89A9-D8A938A40D38}">
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="65.7109375" customWidth="1"/>
@@ -762,131 +672,11 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>38</v>
-      </c>
-      <c r="B20" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>40</v>
-      </c>
-      <c r="B21" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>44</v>
-      </c>
-      <c r="B23" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>46</v>
-      </c>
-      <c r="B24" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>48</v>
-      </c>
-      <c r="B25" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>50</v>
-      </c>
-      <c r="B26" t="s">
-        <v>51</v>
-      </c>
-    </row>
   </sheetData>
   <conditionalFormatting sqref="B3">
     <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B9">
+  <conditionalFormatting sqref="B5">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Moved the replace step outside the with ZipFile(...) block so the file handle is closed before files are swapped
</commit_message>
<xml_diff>
--- a/CustomField_LookupTable.xlsx
+++ b/CustomField_LookupTable.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft5071812-my.sharepoint.com/personal/tdolan_quillarrowlaw_com/Documents/Documents/ClioTemplates_CustomFields_MassUpdate/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="329" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB76B858-04F5-4F69-8B88-067FEBBA2A04}"/>
+  <xr:revisionPtr revIDLastSave="339" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88743A12-1F92-4173-9B6C-682D8E706A3C}"/>
   <bookViews>
-    <workbookView xWindow="7230" yWindow="1695" windowWidth="18570" windowHeight="13680" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
+    <workbookView xWindow="31245" yWindow="1155" windowWidth="18570" windowHeight="13680" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
   </bookViews>
   <sheets>
     <sheet name="LookupTable" sheetId="1" r:id="rId1"/>
@@ -47,61 +47,61 @@
     <t>&lt;&lt; date.verbose &gt;&gt;</t>
   </si>
   <si>
-    <t>&lt;&lt; date.verbose _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
     <t>&lt;&lt; matter.customfield.casenumber &gt;&gt;</t>
   </si>
   <si>
-    <t>&lt;&lt; matter.customfield.casenumber _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
     <t>&lt;&lt; matter.customfield.county &gt;&gt;</t>
   </si>
   <si>
-    <t>&lt;&lt; matter.customfield.county _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
     <t>&lt;&lt; matter.customfield.judge &gt;&gt;</t>
   </si>
   <si>
-    <t>&lt;&lt; matter.customfield.judge _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
     <t>&lt;&lt; matter.customfield.occitystatezip &gt;&gt;</t>
   </si>
   <si>
-    <t>&lt;&lt; matter.customfield.occitystatezip _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
     <t>&lt;&lt; matter.customfield.ocfirmname &gt;&gt;</t>
   </si>
   <si>
-    <t>&lt;&lt; matter.customfield.ocfirmname _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
     <t>&lt;&lt; matter.customfield.ocname1 &gt;&gt;</t>
   </si>
   <si>
-    <t>&lt;&lt; matter.customfield.ocname1 _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
     <t>&lt;&lt; matter.customfield.ocname2 &gt;&gt;</t>
   </si>
   <si>
-    <t>&lt;&lt; matter.customfield.ocname2 _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
     <t>&lt;&lt; matter.customfield.ocstreetaddress &gt;&gt;</t>
   </si>
   <si>
-    <t>&lt;&lt; matter.customfield.ocstreetaddress _UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
     <t>&lt;&lt; matter.customfield.plaintiffsfulllegalname &gt;&gt;</t>
   </si>
   <si>
-    <t>&lt;&lt; matter.customfield.plaintiffsfulllegalname _UPDATED_031126 &gt;&gt;</t>
+    <t>&lt;&lt; matter.customfield.casenumber_UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.county_UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.judge_UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.occitystatezip_UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.ocfirmname_UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.ocname1_UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.ocname2_UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.ocstreetaddress_UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.plaintiffsfulllegalname_UPDATED_031126 &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; date.verbose_UPDATED_031126 &gt;&gt;</t>
   </si>
 </sst>
 </file>
@@ -597,68 +597,68 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
         <v>19</v>
@@ -666,10 +666,10 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
         <v>20</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated clio_templates_sync.py to include the xml_replace_templates.py script to replace the placeholders inside the docx XML (word/*.xml), which captures text box content for testing
</commit_message>
<xml_diff>
--- a/CustomField_LookupTable.xlsx
+++ b/CustomField_LookupTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft5071812-my.sharepoint.com/personal/tdolan_quillarrowlaw_com/Documents/Documents/ClioTemplates_CustomFields_MassUpdate/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="339" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{88743A12-1F92-4173-9B6C-682D8E706A3C}"/>
+  <xr:revisionPtr revIDLastSave="360" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA5C8A54-4B68-4235-8EDA-F07E5E5AD5CA}"/>
   <bookViews>
-    <workbookView xWindow="31245" yWindow="1155" windowWidth="18570" windowHeight="13680" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
+    <workbookView xWindow="3360" yWindow="1020" windowWidth="23010" windowHeight="13650" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
   </bookViews>
   <sheets>
     <sheet name="LookupTable" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
   <si>
     <t>New_Value</t>
   </si>
@@ -53,62 +53,35 @@
     <t>&lt;&lt; matter.customfield.county &gt;&gt;</t>
   </si>
   <si>
-    <t>&lt;&lt; matter.customfield.judge &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.occitystatezip &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.ocfirmname &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.ocname1 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.ocname2 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.ocstreetaddress &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.plaintiffsfulllegalname &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.casenumber_UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.county_UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.judge_UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.occitystatezip_UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.ocfirmname_UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.ocname1_UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.ocname2_UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.ocstreetaddress_UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.plaintiffsfulllegalname_UPDATED_031126 &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; date.verbose_UPDATED_031126 &gt;&gt;</t>
+    <t>&lt;&lt; Matter.CustomField.DefendantsNameShort &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; date.verbose_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.casenumber_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.county_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; TestCustomField.Test &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; TestCustomField.Test_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.VehicleYear &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.VehicleYearTESTUPDATE &gt;&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -123,6 +96,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -145,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -153,21 +132,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -251,11 +221,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}" name="Table1" displayName="Table1" ref="A1:B11" totalsRowShown="0" headerRowDxfId="4">
-  <autoFilter ref="A1:B11" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}" name="Table1" displayName="Table1" ref="A1:B7" totalsRowShown="0" headerRowDxfId="3">
+  <autoFilter ref="A1:B7" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{52BB13A1-40AB-4518-B0DE-62637CB7D74A}" name="Old_Value" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{06BCDB60-C4F4-4E5F-B692-5B8737E55DE6}" name="New_Value" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{52BB13A1-40AB-4518-B0DE-62637CB7D74A}" name="Old_Value" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{06BCDB60-C4F4-4E5F-B692-5B8737E55DE6}" name="New_Value" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -578,7 +548,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAF23435-C8D7-4BEB-89A9-D8A938A40D38}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="65.7109375" customWidth="1"/>
@@ -597,7 +567,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -605,7 +575,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -613,7 +583,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -621,63 +591,28 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="A7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B9" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="B7" s="3" t="s">
         <v>10</v>
-      </c>
-      <c r="B10" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>11</v>
-      </c>
-      <c r="B11" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B3">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B5">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Updated apply_xml_replacements() function in mass_update_templates.py to replace the placeholders inside the docx XML (word/*.xml), which captures text box content for testing
</commit_message>
<xml_diff>
--- a/CustomField_LookupTable.xlsx
+++ b/CustomField_LookupTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft5071812-my.sharepoint.com/personal/tdolan_quillarrowlaw_com/Documents/Documents/ClioTemplates_CustomFields_MassUpdate/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="360" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA5C8A54-4B68-4235-8EDA-F07E5E5AD5CA}"/>
+  <xr:revisionPtr revIDLastSave="374" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7DFA38D-8D86-4448-8947-7F8F6D8C93D5}"/>
   <bookViews>
-    <workbookView xWindow="3360" yWindow="1020" windowWidth="23010" windowHeight="13650" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
+    <workbookView xWindow="30675" yWindow="1215" windowWidth="23010" windowHeight="13650" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
   </bookViews>
   <sheets>
     <sheet name="LookupTable" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>New_Value</t>
   </si>
@@ -44,37 +44,40 @@
     <t>Old_Value</t>
   </si>
   <si>
-    <t>&lt;&lt; date.verbose &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.casenumber &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.county &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.DefendantsNameShort &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; date.verbose_TESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.casenumber_TESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.county_TESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; TestCustomField.Test &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; TestCustomField.Test_TESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.VehicleYear &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.VehicleYearTESTUPDATE &gt;&gt;</t>
+    <t>date.verbose</t>
+  </si>
+  <si>
+    <t>matter.customfield.casenumber</t>
+  </si>
+  <si>
+    <t>matter.customfield.county</t>
+  </si>
+  <si>
+    <t>Matter.CustomField.DefendantsNameShort</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Matter.CustomField.VehicleYear</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> TestCustomField.Test</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> date.verbose_TESTUPDATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> matter.customfield.casenumber_TESTUPDATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> matter.customfield.county_TESTUPDATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Matter.CustomField.DefendantsNameShort</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Matter.CustomField.VehicleYearTESTUPDATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> TestCustomField.Test_TESTUPDATE</t>
   </si>
 </sst>
 </file>
@@ -567,7 +570,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -575,7 +578,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -583,7 +586,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -591,12 +594,12 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
         <v>12</v>
@@ -604,10 +607,10 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated mass_update_templates.py to have more efficient XML replacement logic and updated .gitignore to ignore CustomField_LookupTable.xlsx
</commit_message>
<xml_diff>
--- a/CustomField_LookupTable.xlsx
+++ b/CustomField_LookupTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft5071812-my.sharepoint.com/personal/tdolan_quillarrowlaw_com/Documents/Documents/ClioTemplates_CustomFields_MassUpdate/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="374" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7DFA38D-8D86-4448-8947-7F8F6D8C93D5}"/>
+  <xr:revisionPtr revIDLastSave="449" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A362E661-6DDE-41E4-AD3B-EF7EC3ED998D}"/>
   <bookViews>
-    <workbookView xWindow="30675" yWindow="1215" windowWidth="23010" windowHeight="13650" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
   </bookViews>
   <sheets>
     <sheet name="LookupTable" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
   <si>
     <t>New_Value</t>
   </si>
@@ -44,40 +44,37 @@
     <t>Old_Value</t>
   </si>
   <si>
-    <t>date.verbose</t>
-  </si>
-  <si>
-    <t>matter.customfield.casenumber</t>
-  </si>
-  <si>
-    <t>matter.customfield.county</t>
-  </si>
-  <si>
-    <t>Matter.CustomField.DefendantsNameShort</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Matter.CustomField.VehicleYear</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> TestCustomField.Test</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> date.verbose_TESTUPDATE</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> matter.customfield.casenumber_TESTUPDATE</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> matter.customfield.county_TESTUPDATE</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Matter.CustomField.DefendantsNameShort</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Matter.CustomField.VehicleYearTESTUPDATE</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> TestCustomField.Test_TESTUPDATE</t>
+    <t>&lt;&lt; date.verbose &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.casenumber &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.county &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.DefendantsNameShort &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.VehicleYear &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; TestCustomField.Test &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; date.verbose_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.casenumber_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.county_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.VehicleYearTESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt;  TestCustomField.Test_TESTUPDATE &gt;&gt;</t>
   </si>
 </sst>
 </file>
@@ -142,16 +139,6 @@
   </cellStyles>
   <dxfs count="4">
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left style="medium">
@@ -206,6 +193,16 @@
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -224,11 +221,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}" name="Table1" displayName="Table1" ref="A1:B7" totalsRowShown="0" headerRowDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}" name="Table1" displayName="Table1" ref="A1:B7" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="A1:B7" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{52BB13A1-40AB-4518-B0DE-62637CB7D74A}" name="Old_Value" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{06BCDB60-C4F4-4E5F-B692-5B8737E55DE6}" name="New_Value" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{52BB13A1-40AB-4518-B0DE-62637CB7D74A}" name="Old_Value" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{06BCDB60-C4F4-4E5F-B692-5B8737E55DE6}" name="New_Value" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -594,7 +591,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -602,7 +599,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -610,12 +607,12 @@
         <v>7</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B3">
-    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
XML replacement now operates on raw XML text nodes (preserves structure), XML pass ignores mc:Fallback to prevent double counts, and updated CHANGELOG_2026-02-03.txt and CustomField_LookupTable.xlsx
</commit_message>
<xml_diff>
--- a/CustomField_LookupTable.xlsx
+++ b/CustomField_LookupTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft5071812-my.sharepoint.com/personal/tdolan_quillarrowlaw_com/Documents/Documents/ClioTemplates_CustomFields_MassUpdate/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="449" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A362E661-6DDE-41E4-AD3B-EF7EC3ED998D}"/>
+  <xr:revisionPtr revIDLastSave="463" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86B43FD7-A487-41BE-9C06-C82953C4115F}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
+    <workbookView xWindow="33735" yWindow="1575" windowWidth="23010" windowHeight="13650" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
   </bookViews>
   <sheets>
     <sheet name="LookupTable" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>New_Value</t>
   </si>
@@ -71,17 +71,32 @@
     <t>&lt;&lt; matter.customfield.county_TESTUPDATE &gt;&gt;</t>
   </si>
   <si>
-    <t>&lt;&lt; Matter.CustomField.VehicleYearTESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
     <t>&lt;&lt;  TestCustomField.Test_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.CourtStreetAddress &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.CaseNameShort &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.CaseNameShort_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.CourtStreetAddress_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.DefendantsNameShort_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.VehicleYear_TESTUPDATE &gt;&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -96,12 +111,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -124,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -132,12 +141,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
+  <dxfs count="3">
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
@@ -193,16 +201,6 @@
       </font>
       <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -221,8 +219,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}" name="Table1" displayName="Table1" ref="A1:B7" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="A1:B7" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}" name="Table1" displayName="Table1" ref="A1:B9" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:B9" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{52BB13A1-40AB-4518-B0DE-62637CB7D74A}" name="Old_Value" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{06BCDB60-C4F4-4E5F-B692-5B8737E55DE6}" name="New_Value" dataDxfId="0"/>
@@ -548,7 +546,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAF23435-C8D7-4BEB-89A9-D8A938A40D38}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="65.7109375" customWidth="1"/>
@@ -591,7 +589,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -599,21 +597,34 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="B3">
-    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
Added a new folder to the gitignore file to ignore the Testing_Files folder
</commit_message>
<xml_diff>
--- a/CustomField_LookupTable.xlsx
+++ b/CustomField_LookupTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft5071812-my.sharepoint.com/personal/tdolan_quillarrowlaw_com/Documents/Documents/ClioTemplates_CustomFields_MassUpdate/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="463" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{86B43FD7-A487-41BE-9C06-C82953C4115F}"/>
+  <xr:revisionPtr revIDLastSave="465" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E16D0CF-0D47-4D5E-83F2-F017E09E9AB3}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
   </bookViews>
   <sheets>
     <sheet name="LookupTable" sheetId="1" r:id="rId1"/>
@@ -59,9 +59,6 @@
     <t>&lt;&lt; Matter.CustomField.VehicleYear &gt;&gt;</t>
   </si>
   <si>
-    <t>&lt;&lt; TestCustomField.Test &gt;&gt;</t>
-  </si>
-  <si>
     <t>&lt;&lt; date.verbose_TESTUPDATE &gt;&gt;</t>
   </si>
   <si>
@@ -71,9 +68,6 @@
     <t>&lt;&lt; matter.customfield.county_TESTUPDATE &gt;&gt;</t>
   </si>
   <si>
-    <t>&lt;&lt;  TestCustomField.Test_TESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
     <t>&lt;&lt; Matter.CustomField.CourtStreetAddress &gt;&gt;</t>
   </si>
   <si>
@@ -90,6 +84,12 @@
   </si>
   <si>
     <t>&lt;&lt; Matter.CustomField.VehicleYear_TESTUPDATE &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Test.CustomField &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Test.CustomField_TESTUPDATE &gt;&gt;</t>
   </si>
 </sst>
 </file>
@@ -565,7 +565,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -573,7 +573,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -581,7 +581,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -589,7 +589,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -597,31 +597,31 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated the .venv/.gitignore file to ignore the clio_templates_manifest.json, clio_tokens.json, custom_field_inventory.xlsx, replacement_report.csv, verification_report.csv, CustomField_LookupTable.xlsx, and xml_debug_log.csv files
</commit_message>
<xml_diff>
--- a/CustomField_LookupTable.xlsx
+++ b/CustomField_LookupTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft5071812-my.sharepoint.com/personal/tdolan_quillarrowlaw_com/Documents/Documents/ClioTemplates_CustomFields_MassUpdate/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="465" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4E16D0CF-0D47-4D5E-83F2-F017E09E9AB3}"/>
+  <xr:revisionPtr revIDLastSave="475" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B478AE9D-5085-42ED-BC95-883E5CC80AB8}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
   </bookViews>
   <sheets>
     <sheet name="LookupTable" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>New_Value</t>
   </si>
@@ -44,52 +44,28 @@
     <t>Old_Value</t>
   </si>
   <si>
-    <t>&lt;&lt; date.verbose &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.casenumber &gt;&gt;</t>
-  </si>
-  <si>
     <t>&lt;&lt; matter.customfield.county &gt;&gt;</t>
   </si>
   <si>
-    <t>&lt;&lt; Matter.CustomField.DefendantsNameShort &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.VehicleYear &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; date.verbose_TESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.casenumber_TESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.county_TESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.CourtStreetAddress &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.CaseNameShort &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.CaseNameShort_TESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.CourtStreetAddress_TESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.DefendantsNameShort_TESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Matter.CustomField.VehicleYear_TESTUPDATE &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Test.CustomField &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; Test.CustomField_TESTUPDATE &gt;&gt;</t>
+    <t>&lt;&lt; matter.customfield.occitystatezip &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.ocstreetaddress &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.ocfirmname &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.county_UPDATED &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.occitystatezip_UPDATED &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.ocstreetaddress_UPDATED &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; matter.customfield.ocfirmname_UPDATED &gt;&gt;</t>
   </si>
 </sst>
 </file>
@@ -133,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -141,6 +117,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -219,8 +196,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}" name="Table1" displayName="Table1" ref="A1:B9" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="A1:B9" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}" name="Table1" displayName="Table1" ref="A1:B5" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:B5" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{52BB13A1-40AB-4518-B0DE-62637CB7D74A}" name="Old_Value" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{06BCDB60-C4F4-4E5F-B692-5B8737E55DE6}" name="New_Value" dataDxfId="0"/>
@@ -546,7 +523,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAF23435-C8D7-4BEB-89A9-D8A938A40D38}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="65.7109375" customWidth="1"/>
@@ -561,67 +538,35 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
-        <v>7</v>
+      <c r="B2" s="3" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" t="s">
-        <v>8</v>
+      <c r="B3" s="3" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B4" t="s">
-        <v>9</v>
+      <c r="B4" s="3" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="A5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
+      <c r="B5" s="3" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Bug found in the inventory_custom_fields.py file The script was not including headers and footers in the text extraction Updated the script to include headers and footers in the text extraction
</commit_message>
<xml_diff>
--- a/CustomField_LookupTable.xlsx
+++ b/CustomField_LookupTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://netorgft5071812-my.sharepoint.com/personal/tdolan_quillarrowlaw_com/Documents/Documents/ClioTemplates_CustomFields_MassUpdate/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="475" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B478AE9D-5085-42ED-BC95-883E5CC80AB8}"/>
+  <xr:revisionPtr revIDLastSave="530" documentId="8_{E80BBBE6-58B7-4864-BD78-E0E1CDA502EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF9A57E3-1BE6-40A4-9991-4F05E5F778E1}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
+    <workbookView xWindow="33345" yWindow="2265" windowWidth="18975" windowHeight="12990" xr2:uid="{28124E9B-F57B-404E-A792-64830DDEDE95}"/>
   </bookViews>
   <sheets>
     <sheet name="LookupTable" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
   <si>
     <t>New_Value</t>
   </si>
@@ -44,35 +44,263 @@
     <t>Old_Value</t>
   </si>
   <si>
-    <t>&lt;&lt; matter.customfield.county &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.occitystatezip &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.ocstreetaddress &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.ocfirmname &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.county_UPDATED &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.occitystatezip_UPDATED &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.ocstreetaddress_UPDATED &gt;&gt;</t>
-  </si>
-  <si>
-    <t>&lt;&lt; matter.customfield.ocfirmname_UPDATED &gt;&gt;</t>
+    <t>&lt;&lt; Matter.CustomField.DateOfVehiclePurcahse &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.VehiclePurchaseDate &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.VehicleInspection &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.VehicleInspectionDate &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.CashPriceOfVehicle &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.VehicleCashPrice &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.Surrender &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.Surrendered &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.Cashbb &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.BuybackCalulator &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.WhoSettled &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.CpPortion &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.AmountOfSettlement &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.OscReDismissal &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.PreviousAccident &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.DescriptionOfProblemsros &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.PlaintiffsNameShort &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.PlaintiffsFullLegalName &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.2ndDefendantsNameShort &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.2ndDefendantsFullLegalName &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.2ndDefendantsEntityType &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.StatefederalCourt &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.MtcArbHearing &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.Msj &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.Cmc &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.Answer2ndDef &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.ServicingDealership4Loc &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.ServicingDealership3Loc &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.ServicingDealership2Loc &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.ServicingDealership1Loc &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.InitialDisclosures &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.EneStatementDue &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.DiscoCutoffFed &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.DateRemoved &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.26fReportcmcDueNorthern &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.DateDiscoverySetOneServed &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.DateDiscoSetTwoServed &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.Mediator &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.Mediation &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.ArbitrationInitiationInvDate &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.ArbInitiatedWith &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.AdrStipFiled &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.Msc &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.Fsctrc &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.AttorneyFeeMtnHearingDate &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.Amount &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.CashorBuyback &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.BuybackCalculator &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.SettlementAttorney &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.CPPortionAmount &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.SettlementAmount &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.OSCDismissalDate &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.PriorAccidents &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.Defects &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.PlaintiffNameShort &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.PlaintiffFullLegalName &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.2ndDefendantShortName &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.2ndDefendantFullLegalName &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.2ndDefendantEntityType &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.Jurisdiction &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.MTCArbitrationHearing &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.MSJDate &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.CmcDate &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.Answer2ndDefendant &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.ServicingDealership4Location &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.ServicingDealership3Location &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.ServicingDealership2Location &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.ServicingDealership1Location &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.FederalInitialDisclosures &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.PlaintiffENEStatementDue &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.FactDiscoveryCutoff &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.RemovalDate &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.Rule26fReportorCMCDue &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.DiscoverySet1Served &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.DiscoverySet2Served &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.MediatorName &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.MediationDate &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.ArbitrationInitiationDate &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.ArbitrationInitiatedWith &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.ADRStipulationFiled &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.MSCDate &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.PreTrialDate &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.AttorneyFeeMotionHearingDate &gt;&gt;</t>
+  </si>
+  <si>
+    <t>&lt;&lt; Matter.CustomField.BuybackAmount &gt;&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -88,13 +316,31 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBEFF1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -117,47 +363,43 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="3">
     <dxf>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
+      <font>
+        <sz val="10"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFEBEFF1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="medium">
-          <color indexed="64"/>
-        </left>
-        <right style="medium">
-          <color indexed="64"/>
-        </right>
-        <top/>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
+      <font>
+        <sz val="10"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFEBEFF1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -196,8 +438,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}" name="Table1" displayName="Table1" ref="A1:B5" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="A1:B5" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}" name="Table1" displayName="Table1" ref="A1:B43" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:B43" xr:uid="{6CDBC208-8FF6-478D-95B6-188E225F38B1}"/>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{52BB13A1-40AB-4518-B0DE-62637CB7D74A}" name="Old_Value" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{06BCDB60-C4F4-4E5F-B692-5B8737E55DE6}" name="New_Value" dataDxfId="0"/>
@@ -523,7 +765,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AAF23435-C8D7-4BEB-89A9-D8A938A40D38}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="65.7109375" customWidth="1"/>
@@ -539,37 +781,342 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>6</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>7</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>8</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B33" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>9</v>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B42" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>